<commit_message>
Eintritte, Kiosk und Spezpreis für Film Veuve Clicquot
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37392E8A-B0F7-42C2-9660-F40DD9B3C67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F91A4F8-C71F-4639-ABC8-76FC039A6314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6720" yWindow="3180" windowWidth="15684" windowHeight="11832" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="2040" yWindow="4020" windowWidth="15684" windowHeight="11832" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="54">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -192,6 +192,15 @@
   </si>
   <si>
     <t>98 85900 00000 00000 00009 17792</t>
+  </si>
+  <si>
+    <t>1020.521</t>
+  </si>
+  <si>
+    <t>Champagner Einkauf: Veuve Clicquot</t>
+  </si>
+  <si>
+    <t>Stefan Jablonski</t>
   </si>
 </sst>
 </file>
@@ -283,20 +292,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -313,10 +318,10 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -367,23 +372,23 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K8" totalsRowShown="0">
-  <autoFilter ref="A1:K8" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K9" totalsRowShown="0">
+  <autoFilter ref="A1:K9" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K4">
     <sortCondition ref="A1:A4"/>
   </sortState>
   <tableColumns count="11">
     <tableColumn id="9" xr3:uid="{7720D0EA-5763-4F4F-82DA-8D34884933A7}" name="Kategorie"/>
     <tableColumn id="8" xr3:uid="{12477251-A7BF-41F7-9734-91E55C44981E}" name="Spieldatum" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{90784966-A7C8-41A3-8EC0-117CDC7DFB09}" name="Suisanummer" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{90784966-A7C8-41A3-8EC0-117CDC7DFB09}" name="Suisanummer" dataDxfId="0"/>
     <tableColumn id="1" xr3:uid="{CADC5726-010C-420F-B3D1-E5B1B323B7D4}" name="Bezeichnung"/>
-    <tableColumn id="2" xr3:uid="{48234371-EC10-4470-8D2A-22FC4E54CF28}" name="Datum" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{90883362-F5C5-4472-9591-164F8C364C6F}" name="Betrag" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{48234371-EC10-4470-8D2A-22FC4E54CF28}" name="Datum" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{90883362-F5C5-4472-9591-164F8C364C6F}" name="Betrag" dataDxfId="4"/>
     <tableColumn id="4" xr3:uid="{0C538012-5D92-4E64-B81F-85CAF66FE963}" name="Firmennamen"/>
     <tableColumn id="5" xr3:uid="{528DBE91-75A0-4B49-8AC8-06D027A50035}" name="Adresse"/>
-    <tableColumn id="6" xr3:uid="{4B5E1481-D849-49CA-8C98-0F7393B356B7}" name="Referenz" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{64D50181-342C-4387-875F-8ADB060C0EDC}" name="Rechnungsnummer" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{9B01639A-96D8-4A50-B1D3-C69E9C49B9DA}" name="Buchungskonto" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{4B5E1481-D849-49CA-8C98-0F7393B356B7}" name="Referenz" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{64D50181-342C-4387-875F-8ADB060C0EDC}" name="Rechnungsnummer" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{9B01639A-96D8-4A50-B1D3-C69E9C49B9DA}" name="Buchungskonto" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -774,7 +779,7 @@
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="45.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
@@ -792,7 +797,7 @@
       <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D1" t="s">
@@ -990,42 +995,66 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="1">
         <v>45667</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" t="s">
         <v>47</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="1">
         <v>45694</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="3">
         <v>121</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" t="s">
         <v>48</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" t="s">
         <v>49</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="12">
+      <c r="J8" s="2">
         <v>91779</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="K8" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F9" s="3"/>
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="1">
+        <v>45701</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="1">
+        <v>45698</v>
+      </c>
+      <c r="F9" s="3">
+        <f>3*54.9</f>
+        <v>164.7</v>
+      </c>
+      <c r="G9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F10" s="3"/>
@@ -1351,7 +1380,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{551055D3-EB54-4023-842C-CF79CAE47FBC}">
           <x14:formula1>
             <xm:f>dropdown!$A$2:$A$8</xm:f>

</xml_diff>

<commit_message>
Verleiherrechung+Spez preise seed of sacred fig
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F91A4F8-C71F-4639-ABC8-76FC039A6314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD58BC5-F114-4B6F-9EE4-CF5A490DB853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2040" yWindow="4020" windowWidth="15684" windowHeight="11832" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="2388" yWindow="4368" windowWidth="15684" windowHeight="11832" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="60">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -201,6 +201,24 @@
   </si>
   <si>
     <t>Stefan Jablonski</t>
+  </si>
+  <si>
+    <t>1020.599</t>
+  </si>
+  <si>
+    <t>Film: The Seed of the sacred fig</t>
+  </si>
+  <si>
+    <t>trigon-film</t>
+  </si>
+  <si>
+    <t>Limmatauweg 9, 5408 Ennetbaden</t>
+  </si>
+  <si>
+    <t>00 00000 00000 00000 04400 59099</t>
+  </si>
+  <si>
+    <t>44005909</t>
   </si>
 </sst>
 </file>
@@ -318,13 +336,13 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;CHF&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -372,23 +390,23 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K9" totalsRowShown="0">
-  <autoFilter ref="A1:K9" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K11" totalsRowShown="0">
+  <autoFilter ref="A1:K11" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K4">
     <sortCondition ref="A1:A4"/>
   </sortState>
   <tableColumns count="11">
     <tableColumn id="9" xr3:uid="{7720D0EA-5763-4F4F-82DA-8D34884933A7}" name="Kategorie"/>
     <tableColumn id="8" xr3:uid="{12477251-A7BF-41F7-9734-91E55C44981E}" name="Spieldatum" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{90784966-A7C8-41A3-8EC0-117CDC7DFB09}" name="Suisanummer" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{90784966-A7C8-41A3-8EC0-117CDC7DFB09}" name="Suisanummer" dataDxfId="5"/>
     <tableColumn id="1" xr3:uid="{CADC5726-010C-420F-B3D1-E5B1B323B7D4}" name="Bezeichnung"/>
-    <tableColumn id="2" xr3:uid="{48234371-EC10-4470-8D2A-22FC4E54CF28}" name="Datum" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{90883362-F5C5-4472-9591-164F8C364C6F}" name="Betrag" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{48234371-EC10-4470-8D2A-22FC4E54CF28}" name="Datum" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{90883362-F5C5-4472-9591-164F8C364C6F}" name="Betrag" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{0C538012-5D92-4E64-B81F-85CAF66FE963}" name="Firmennamen"/>
     <tableColumn id="5" xr3:uid="{528DBE91-75A0-4B49-8AC8-06D027A50035}" name="Adresse"/>
-    <tableColumn id="6" xr3:uid="{4B5E1481-D849-49CA-8C98-0F7393B356B7}" name="Referenz" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{64D50181-342C-4387-875F-8ADB060C0EDC}" name="Rechnungsnummer" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{9B01639A-96D8-4A50-B1D3-C69E9C49B9DA}" name="Buchungskonto" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{4B5E1481-D849-49CA-8C98-0F7393B356B7}" name="Referenz" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{64D50181-342C-4387-875F-8ADB060C0EDC}" name="Rechnungsnummer" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{9B01639A-96D8-4A50-B1D3-C69E9C49B9DA}" name="Buchungskonto" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1057,10 +1075,46 @@
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F10" s="3"/>
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="1">
+        <v>45683</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="1">
+        <v>45701</v>
+      </c>
+      <c r="F10" s="3">
+        <v>194.6</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E11" s="1"/>
       <c r="F11" s="3"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="F12" s="3"/>

</xml_diff>

<commit_message>
Rechnungen, Veuve Clicquot, Missile, der Vierer und Mitgliederbeitrag SKV
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BD58BC5-F114-4B6F-9EE4-CF5A490DB853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6790A8-FD22-4AF7-85B4-8652BC0D60A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2388" yWindow="4368" windowWidth="15684" windowHeight="11832" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="14580" windowHeight="17370" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="80">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -219,6 +219,66 @@
   </si>
   <si>
     <t>44005909</t>
+  </si>
+  <si>
+    <t>1020.428</t>
+  </si>
+  <si>
+    <t>Film: The Missile</t>
+  </si>
+  <si>
+    <t>Frenetic Films Ag</t>
+  </si>
+  <si>
+    <t>Riedtlistrasse 23, 8006 Zürich</t>
+  </si>
+  <si>
+    <t>26 27680 00000 00000 01005 44245</t>
+  </si>
+  <si>
+    <t>SKV Mitgliederbeitrag</t>
+  </si>
+  <si>
+    <t>Schweizerischer Kino-Verband</t>
+  </si>
+  <si>
+    <t>Theaterstrasse 10, 8001 Zürich</t>
+  </si>
+  <si>
+    <t>14718</t>
+  </si>
+  <si>
+    <t>1020.652</t>
+  </si>
+  <si>
+    <t>Film: Der Vierer</t>
+  </si>
+  <si>
+    <t>DCM Film Distribution (Schweiz) GmbH</t>
+  </si>
+  <si>
+    <t>Kreuzstrasse 2, 8008 Zürich</t>
+  </si>
+  <si>
+    <t>96 57660 00000 00000 00302 33275</t>
+  </si>
+  <si>
+    <t>03023327</t>
+  </si>
+  <si>
+    <t>Film: Veuve Clicqot</t>
+  </si>
+  <si>
+    <t>Praesens Film Ag</t>
+  </si>
+  <si>
+    <t>Münchhaldenstrasse 19, 8008 Zürich</t>
+  </si>
+  <si>
+    <t>00 00000 00000 00000 00004 48020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00044802 </t>
   </si>
 </sst>
 </file>
@@ -390,8 +450,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K11" totalsRowShown="0">
-  <autoFilter ref="A1:K11" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K14" totalsRowShown="0">
+  <autoFilter ref="A1:K14" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K4">
     <sortCondition ref="A1:A4"/>
   </sortState>
@@ -733,18 +793,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A72045E-24F3-4DFF-AD02-E9648BA6850D}">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" customWidth="1"/>
-    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.44140625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.36328125" customWidth="1"/>
+    <col min="2" max="2" width="37.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.453125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="13.08984375" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="42.44140625" customWidth="1"/>
+    <col min="8" max="8" width="42.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -793,22 +853,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D174BE7-BB11-4664-AEC1-AB301D6C9797}">
   <dimension ref="A1:L114"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="45.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="45.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31" customWidth="1"/>
-    <col min="8" max="8" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.6640625" customWidth="1"/>
+    <col min="8" max="8" width="35.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -843,7 +903,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -868,7 +928,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -892,7 +952,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -915,7 +975,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -944,7 +1004,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -977,7 +1037,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1012,7 +1072,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1047,7 +1107,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1074,7 +1134,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1109,320 +1169,434 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="E11" s="1"/>
-      <c r="F11" s="3"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F12" s="3"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F13" s="3"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1">
+        <v>45689</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="1">
+        <v>45707</v>
+      </c>
+      <c r="F11" s="3">
+        <v>214.05</v>
+      </c>
+      <c r="G11" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J11">
+        <v>10054424</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="1">
+        <v>45709</v>
+      </c>
+      <c r="F12" s="3">
+        <v>100</v>
+      </c>
+      <c r="G12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="K12" s="2"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="1">
+        <v>45695</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" s="1">
+        <v>45717</v>
+      </c>
+      <c r="F13" s="3">
+        <v>194.6</v>
+      </c>
+      <c r="G13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H13" t="s">
+        <v>72</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="1">
+        <v>45701</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" s="1">
+        <v>45707</v>
+      </c>
+      <c r="F14" s="3">
+        <v>142.05000000000001</v>
+      </c>
+      <c r="G14" t="s">
+        <v>76</v>
+      </c>
+      <c r="H14" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F101" s="3"/>
     </row>
-    <row r="102" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F102" s="3"/>
     </row>
-    <row r="103" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F103" s="3"/>
     </row>
-    <row r="104" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F104" s="3"/>
     </row>
-    <row r="105" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F105" s="3"/>
     </row>
-    <row r="106" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F106" s="3"/>
     </row>
-    <row r="107" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F107" s="3"/>
     </row>
-    <row r="108" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F108" s="3"/>
     </row>
-    <row r="109" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F109" s="3"/>
     </row>
-    <row r="110" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F110" s="3"/>
     </row>
-    <row r="111" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F111" s="3"/>
     </row>
-    <row r="112" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F112" s="3"/>
     </row>
-    <row r="113" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F113" s="3"/>
     </row>
-    <row r="114" spans="6:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F114" s="3"/>
     </row>
   </sheetData>
@@ -1456,48 +1630,48 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EFEBA5D-FF22-4032-BB29-794CF56A632B}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1513,32 +1687,32 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7625BC9-72E3-4F2B-8D7E-DECECAE27301}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>34</v>
       </c>

</xml_diff>

<commit_message>
Rechnung Harold und die Zauberkreide
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B412A982-D5B2-4876-9D39-F10A8CA42364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7674F76D-9547-45AE-9862-FCC0B7B559E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1344" yWindow="3324" windowWidth="15684" windowHeight="11832" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="1480" yWindow="1480" windowWidth="15100" windowHeight="12710" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="345">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -1067,6 +1067,12 @@
   </si>
   <si>
     <t>Rechnung 136 / 2024</t>
+  </si>
+  <si>
+    <t>Film: Harald und die Zauberkreide</t>
+  </si>
+  <si>
+    <t>3064319</t>
   </si>
 </sst>
 </file>
@@ -1268,8 +1274,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K121" totalsRowShown="0">
-  <autoFilter ref="A1:K121" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K122" totalsRowShown="0">
+  <autoFilter ref="A1:K122" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A9:K113">
     <sortCondition ref="D2:D119"/>
     <sortCondition ref="C2:C119"/>
@@ -1602,18 +1608,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A72045E-24F3-4DFF-AD02-E9648BA6850D}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" customWidth="1"/>
-    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.36328125" customWidth="1"/>
+    <col min="2" max="2" width="37.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.453125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="13.08984375" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="40" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="36" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="42.44140625" customWidth="1"/>
+    <col min="7" max="7" width="42.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1636,7 +1642,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1653,7 +1659,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -1673,7 +1679,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1690,7 +1696,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1707,7 +1713,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1724,7 +1730,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1744,7 +1750,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1761,7 +1767,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -1778,7 +1784,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1795,7 +1801,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -1812,7 +1818,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -1829,7 +1835,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1849,7 +1855,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1872,7 +1878,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1895,7 +1901,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1918,7 +1924,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1941,7 +1947,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -1964,7 +1970,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -1984,7 +1990,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -2030,22 +2036,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D174BE7-BB11-4664-AEC1-AB301D6C9797}">
   <dimension ref="A1:M217"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
-    <col min="7" max="7" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" customWidth="1"/>
-    <col min="11" max="11" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.6328125" customWidth="1"/>
+    <col min="11" max="11" width="16.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -2080,7 +2086,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2106,7 +2112,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -2129,7 +2135,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>73</v>
       </c>
@@ -2160,7 +2166,7 @@
       <c r="L4" s="20"/>
       <c r="M4" s="20"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -2187,7 +2193,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -2218,7 +2224,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -2242,7 +2248,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2268,7 +2274,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2293,7 +2299,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -2317,7 +2323,7 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -2343,7 +2349,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -2374,7 +2380,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -2397,7 +2403,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -2421,7 +2427,7 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -2447,7 +2453,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -2478,7 +2484,7 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -2506,7 +2512,7 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -2537,7 +2543,7 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>73</v>
       </c>
@@ -2564,7 +2570,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -2592,7 +2598,7 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -2615,7 +2621,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -2643,7 +2649,7 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -2664,7 +2670,7 @@
       </c>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -2695,7 +2701,7 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2719,7 +2725,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>15</v>
       </c>
@@ -2742,7 +2748,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>22</v>
       </c>
@@ -2775,7 +2781,7 @@
       <c r="L27" s="20"/>
       <c r="M27" s="20"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>17</v>
       </c>
@@ -2802,7 +2808,7 @@
       <c r="L28" s="6"/>
       <c r="M28" s="6"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>24</v>
       </c>
@@ -2828,7 +2834,7 @@
       <c r="L29" s="20"/>
       <c r="M29" s="20"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>24</v>
       </c>
@@ -2862,7 +2868,7 @@
       <c r="L30" s="20"/>
       <c r="M30" s="20"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>73</v>
       </c>
@@ -2890,7 +2896,7 @@
       <c r="L31" s="20"/>
       <c r="M31" s="20"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>15</v>
       </c>
@@ -2915,7 +2921,7 @@
       <c r="L32" s="20"/>
       <c r="M32" s="20"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>17</v>
       </c>
@@ -2942,7 +2948,7 @@
       <c r="L33" s="20"/>
       <c r="M33" s="20"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>24</v>
       </c>
@@ -2966,7 +2972,7 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>24</v>
       </c>
@@ -2998,7 +3004,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>22</v>
       </c>
@@ -3033,7 +3039,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -3068,7 +3074,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>22</v>
       </c>
@@ -3103,7 +3109,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>22</v>
       </c>
@@ -3138,7 +3144,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>22</v>
       </c>
@@ -3173,7 +3179,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>22</v>
       </c>
@@ -3204,7 +3210,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -3237,7 +3243,7 @@
       </c>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>22</v>
       </c>
@@ -3272,7 +3278,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3305,7 +3311,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>15</v>
       </c>
@@ -3328,7 +3334,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>22</v>
       </c>
@@ -3363,7 +3369,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>17</v>
       </c>
@@ -3388,7 +3394,7 @@
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>24</v>
       </c>
@@ -3412,7 +3418,7 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>22</v>
       </c>
@@ -3443,7 +3449,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>22</v>
       </c>
@@ -3478,7 +3484,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>22</v>
       </c>
@@ -3513,7 +3519,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>22</v>
       </c>
@@ -3546,7 +3552,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>14</v>
       </c>
@@ -3576,7 +3582,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -3606,7 +3612,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>17</v>
       </c>
@@ -3631,7 +3637,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>24</v>
       </c>
@@ -3655,7 +3661,7 @@
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>22</v>
       </c>
@@ -3690,7 +3696,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>24</v>
       </c>
@@ -3722,7 +3728,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>22</v>
       </c>
@@ -3757,7 +3763,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>17</v>
       </c>
@@ -3779,7 +3785,7 @@
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>24</v>
       </c>
@@ -3803,7 +3809,7 @@
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>22</v>
       </c>
@@ -3838,7 +3844,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -3861,7 +3867,7 @@
       <c r="K63" s="2"/>
       <c r="L63" s="6"/>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>17</v>
       </c>
@@ -3886,7 +3892,7 @@
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>24</v>
       </c>
@@ -3910,7 +3916,7 @@
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>24</v>
       </c>
@@ -3942,7 +3948,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>15</v>
       </c>
@@ -3974,7 +3980,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>17</v>
       </c>
@@ -3999,7 +4005,7 @@
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>17</v>
       </c>
@@ -4024,7 +4030,7 @@
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>24</v>
       </c>
@@ -4048,7 +4054,7 @@
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>24</v>
       </c>
@@ -4080,7 +4086,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>15</v>
       </c>
@@ -4103,7 +4109,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>15</v>
       </c>
@@ -4126,7 +4132,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>17</v>
       </c>
@@ -4151,7 +4157,7 @@
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>17</v>
       </c>
@@ -4176,7 +4182,7 @@
       <c r="J75" s="9"/>
       <c r="K75" s="7"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>24</v>
       </c>
@@ -4200,7 +4206,7 @@
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>22</v>
       </c>
@@ -4235,7 +4241,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>24</v>
       </c>
@@ -4267,7 +4273,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>22</v>
       </c>
@@ -4302,7 +4308,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>22</v>
       </c>
@@ -4337,7 +4343,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>73</v>
       </c>
@@ -4360,7 +4366,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>73</v>
       </c>
@@ -4383,7 +4389,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>73</v>
       </c>
@@ -4409,7 +4415,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>73</v>
       </c>
@@ -4432,7 +4438,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>73</v>
       </c>
@@ -4455,7 +4461,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>73</v>
       </c>
@@ -4478,7 +4484,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>73</v>
       </c>
@@ -4513,7 +4519,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>22</v>
       </c>
@@ -4548,7 +4554,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>24</v>
       </c>
@@ -4578,7 +4584,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>15</v>
       </c>
@@ -4601,7 +4607,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>22</v>
       </c>
@@ -4636,7 +4642,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>22</v>
       </c>
@@ -4671,7 +4677,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>17</v>
       </c>
@@ -4696,7 +4702,7 @@
       <c r="J93" s="2"/>
       <c r="K93" s="2"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>17</v>
       </c>
@@ -4721,7 +4727,7 @@
       <c r="J94" s="2"/>
       <c r="K94" s="2"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" s="11" t="s">
         <v>24</v>
       </c>
@@ -4746,7 +4752,7 @@
       <c r="J95" s="18"/>
       <c r="K95" s="19"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>22</v>
       </c>
@@ -4779,7 +4785,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>22</v>
       </c>
@@ -4814,7 +4820,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>22</v>
       </c>
@@ -4849,7 +4855,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>73</v>
       </c>
@@ -4875,7 +4881,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A100" s="10" t="s">
         <v>22</v>
       </c>
@@ -4910,7 +4916,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>22</v>
       </c>
@@ -4945,7 +4951,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>22</v>
       </c>
@@ -4978,7 +4984,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>24</v>
       </c>
@@ -5010,7 +5016,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>17</v>
       </c>
@@ -5035,7 +5041,7 @@
       <c r="J104" s="2"/>
       <c r="K104" s="2"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>17</v>
       </c>
@@ -5060,7 +5066,7 @@
       <c r="J105" s="2"/>
       <c r="K105" s="2"/>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>24</v>
       </c>
@@ -5084,7 +5090,7 @@
       <c r="J106" s="2"/>
       <c r="K106" s="2"/>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>22</v>
       </c>
@@ -5117,7 +5123,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>22</v>
       </c>
@@ -5152,7 +5158,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>15</v>
       </c>
@@ -5184,7 +5190,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>73</v>
       </c>
@@ -5219,7 +5225,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>22</v>
       </c>
@@ -5254,7 +5260,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>17</v>
       </c>
@@ -5279,7 +5285,7 @@
       <c r="J112" s="2"/>
       <c r="K112" s="2"/>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>17</v>
       </c>
@@ -5304,7 +5310,7 @@
       <c r="J113" s="2"/>
       <c r="K113" s="2"/>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>24</v>
       </c>
@@ -5328,7 +5334,7 @@
       <c r="J114" s="2"/>
       <c r="K114" s="2"/>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>22</v>
       </c>
@@ -5363,7 +5369,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>22</v>
       </c>
@@ -5394,7 +5400,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>22</v>
       </c>
@@ -5427,7 +5433,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>14</v>
       </c>
@@ -5455,7 +5461,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>14</v>
       </c>
@@ -5483,7 +5489,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>15</v>
       </c>
@@ -5511,7 +5517,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>22</v>
       </c>
@@ -5544,292 +5550,322 @@
         <v>113</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E122" s="4"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>22</v>
+      </c>
+      <c r="B122" s="1">
+        <v>45599</v>
+      </c>
+      <c r="C122" t="s">
+        <v>343</v>
+      </c>
+      <c r="D122" s="1">
+        <v>45699</v>
+      </c>
+      <c r="E122" s="4">
+        <v>162.5</v>
+      </c>
+      <c r="F122" t="s">
+        <v>307</v>
+      </c>
+      <c r="G122" t="s">
+        <v>43</v>
+      </c>
+      <c r="H122" s="2"/>
+      <c r="I122" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="J122" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="K122" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E123" s="4"/>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E124" s="4"/>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E125" s="4"/>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E126" s="4"/>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E127" s="4"/>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="E128" s="4"/>
     </row>
-    <row r="129" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="129" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E129" s="4"/>
     </row>
-    <row r="130" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="130" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E130" s="4"/>
     </row>
-    <row r="131" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="131" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E131" s="4"/>
     </row>
-    <row r="132" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="132" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E132" s="4"/>
     </row>
-    <row r="133" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="133" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E133" s="4"/>
     </row>
-    <row r="134" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="134" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E134" s="4"/>
     </row>
-    <row r="135" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="135" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E135" s="4"/>
     </row>
-    <row r="136" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="136" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E136" s="4"/>
     </row>
-    <row r="137" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="137" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E137" s="4"/>
     </row>
-    <row r="138" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="138" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E138" s="4"/>
     </row>
-    <row r="139" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="139" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E139" s="4"/>
     </row>
-    <row r="140" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="140" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E140" s="4"/>
     </row>
-    <row r="141" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="141" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E141" s="4"/>
     </row>
-    <row r="142" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="142" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E142" s="4"/>
     </row>
-    <row r="143" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="143" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E143" s="4"/>
     </row>
-    <row r="144" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="144" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E144" s="4"/>
     </row>
-    <row r="145" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="145" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E145" s="4"/>
     </row>
-    <row r="146" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="146" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E146" s="4"/>
     </row>
-    <row r="147" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="147" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E147" s="4"/>
     </row>
-    <row r="148" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="148" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E148" s="4"/>
     </row>
-    <row r="149" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="149" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E149" s="4"/>
     </row>
-    <row r="150" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="150" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E150" s="4"/>
     </row>
-    <row r="151" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="151" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E151" s="4"/>
     </row>
-    <row r="152" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="152" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E152" s="4"/>
     </row>
-    <row r="153" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="153" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E153" s="4"/>
     </row>
-    <row r="154" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="154" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E154" s="4"/>
     </row>
-    <row r="155" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="155" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E155" s="4"/>
     </row>
-    <row r="156" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="156" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E156" s="4"/>
     </row>
-    <row r="157" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="157" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E157" s="4"/>
     </row>
-    <row r="158" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="158" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E158" s="4"/>
     </row>
-    <row r="159" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="159" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E159" s="4"/>
     </row>
-    <row r="160" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="160" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E160" s="4"/>
     </row>
-    <row r="161" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="161" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E161" s="4"/>
     </row>
-    <row r="162" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="162" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E162" s="4"/>
     </row>
-    <row r="163" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="163" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E163" s="4"/>
     </row>
-    <row r="164" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="164" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E164" s="4"/>
     </row>
-    <row r="165" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="165" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E165" s="4"/>
     </row>
-    <row r="166" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="166" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E166" s="4"/>
     </row>
-    <row r="167" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="167" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E167" s="4"/>
     </row>
-    <row r="168" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="168" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E168" s="4"/>
     </row>
-    <row r="169" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="169" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E169" s="4"/>
     </row>
-    <row r="170" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="170" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E170" s="4"/>
     </row>
-    <row r="171" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="171" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E171" s="4"/>
     </row>
-    <row r="172" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="172" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E172" s="4"/>
     </row>
-    <row r="173" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="173" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E173" s="4"/>
     </row>
-    <row r="174" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="174" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E174" s="4"/>
     </row>
-    <row r="175" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="175" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E175" s="4"/>
     </row>
-    <row r="176" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="176" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E176" s="4"/>
     </row>
-    <row r="177" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="177" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E177" s="4"/>
     </row>
-    <row r="178" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="178" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E178" s="4"/>
     </row>
-    <row r="179" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="179" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E179" s="4"/>
     </row>
-    <row r="180" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="180" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E180" s="4"/>
     </row>
-    <row r="181" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="181" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E181" s="4"/>
     </row>
-    <row r="182" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="182" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E182" s="4"/>
     </row>
-    <row r="183" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="183" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E183" s="4"/>
     </row>
-    <row r="184" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="184" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E184" s="4"/>
     </row>
-    <row r="185" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="185" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E185" s="4"/>
     </row>
-    <row r="186" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="186" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E186" s="4"/>
     </row>
-    <row r="187" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="187" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E187" s="4"/>
     </row>
-    <row r="188" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="188" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E188" s="4"/>
     </row>
-    <row r="189" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="189" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E189" s="4"/>
     </row>
-    <row r="190" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="190" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E190" s="4"/>
     </row>
-    <row r="191" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="191" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E191" s="4"/>
     </row>
-    <row r="192" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="192" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E192" s="4"/>
     </row>
-    <row r="193" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="193" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E193" s="4"/>
     </row>
-    <row r="194" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="194" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E194" s="4"/>
     </row>
-    <row r="195" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="195" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E195" s="4"/>
     </row>
-    <row r="196" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="196" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E196" s="4"/>
     </row>
-    <row r="197" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="197" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E197" s="4"/>
     </row>
-    <row r="198" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="198" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E198" s="4"/>
     </row>
-    <row r="199" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="199" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E199" s="4"/>
     </row>
-    <row r="200" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="200" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E200" s="4"/>
     </row>
-    <row r="201" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="201" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E201" s="4"/>
     </row>
-    <row r="202" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="202" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E202" s="4"/>
     </row>
-    <row r="203" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="203" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E203" s="4"/>
     </row>
-    <row r="204" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="204" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E204" s="4"/>
     </row>
-    <row r="205" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="205" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E205" s="4"/>
     </row>
-    <row r="206" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="206" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E206" s="4"/>
     </row>
-    <row r="207" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="207" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E207" s="4"/>
     </row>
-    <row r="208" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="208" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E208" s="4"/>
     </row>
-    <row r="209" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="209" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E209" s="4"/>
     </row>
-    <row r="210" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="210" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E210" s="4"/>
     </row>
-    <row r="211" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="211" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E211" s="4"/>
     </row>
-    <row r="212" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="212" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E212" s="4"/>
     </row>
-    <row r="213" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="213" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E213" s="4"/>
     </row>
-    <row r="214" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="214" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E214" s="4"/>
     </row>
-    <row r="215" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="215" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E215" s="4"/>
     </row>
-    <row r="216" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="216" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E216" s="4"/>
     </row>
-    <row r="217" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="217" spans="5:5" x14ac:dyDescent="0.35">
       <c r="E217" s="4"/>
     </row>
   </sheetData>
@@ -5865,47 +5901,47 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EFEBA5D-FF22-4032-BB29-794CF56A632B}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Neue Rechnung: SKV Akonto1 Suisa
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6790A8-FD22-4AF7-85B4-8652BC0D60A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221D1492-7DE7-4ECC-B250-44282DE7A778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="14580" windowHeight="17370" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="82">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -279,6 +279,12 @@
   </si>
   <si>
     <t xml:space="preserve">00044802 </t>
+  </si>
+  <si>
+    <t>SKV Akonto 1 Suisa</t>
+  </si>
+  <si>
+    <t>14948</t>
   </si>
 </sst>
 </file>
@@ -450,8 +456,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K14" totalsRowShown="0">
-  <autoFilter ref="A1:K14" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K15" totalsRowShown="0">
+  <autoFilter ref="A1:K15" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K4">
     <sortCondition ref="A1:A4"/>
   </sortState>
@@ -859,7 +865,7 @@
     <col min="2" max="2" width="13.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.6328125" style="2" customWidth="1"/>
     <col min="4" max="4" width="45.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31" customWidth="1"/>
     <col min="8" max="8" width="35.6328125" bestFit="1" customWidth="1"/>
@@ -1300,7 +1306,31 @@
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="F15" s="3"/>
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" t="s">
+        <v>80</v>
+      </c>
+      <c r="E15" s="1">
+        <v>45715</v>
+      </c>
+      <c r="F15" s="3">
+        <v>63.7</v>
+      </c>
+      <c r="G15" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" t="s">
+        <v>67</v>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="F16" s="3"/>

</xml_diff>

<commit_message>
Eintritt und Kiosk bis 6.4.25
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062CE880-E6C7-46DA-AF73-3D0B00426065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8508D3F-D98E-4823-9BC4-2B651D9BB3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="14580" windowHeight="17370" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="14340" yWindow="0" windowWidth="14550" windowHeight="17370" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="90">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -297,6 +297,18 @@
   </si>
   <si>
     <t>Streulistrasse 85, 8032 Zürich</t>
+  </si>
+  <si>
+    <t>1020.928</t>
+  </si>
+  <si>
+    <t>Film: The Substance</t>
+  </si>
+  <si>
+    <t>98 85900 00000 00000 00009 29507</t>
+  </si>
+  <si>
+    <t>00092950</t>
   </si>
 </sst>
 </file>
@@ -468,8 +480,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K16" totalsRowShown="0">
-  <autoFilter ref="A1:K16" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K17" totalsRowShown="0">
+  <autoFilter ref="A1:K17" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K4">
     <sortCondition ref="A1:A4"/>
   </sortState>
@@ -1373,52 +1385,84 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.35">
-      <c r="F17" s="3"/>
-    </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>45731</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="1">
+        <v>45744</v>
+      </c>
+      <c r="F17" s="3">
+        <v>73.349999999999994</v>
+      </c>
+      <c r="G17" t="s">
+        <v>48</v>
+      </c>
+      <c r="H17" t="s">
+        <v>49</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="6:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F32" s="3"/>
     </row>
     <row r="33" spans="6:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Rechnungen in Einnahmen Ausgaben eingetragen
</commit_message>
<xml_diff>
--- a/Input/Einnahmen und Ausgaben.xlsx
+++ b/Input/Einnahmen und Ausgaben.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\R Packages\Kinoklub\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F15EF7-BC82-4503-B6DB-BAF770A8AFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6308EFF3-A270-4FF3-AA2B-4BDC85F316CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="14580" windowHeight="17370" xr2:uid="{D194CBB7-18DA-440A-A6D7-06C22280DEE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Einnahmen" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="118">
   <si>
     <t>Bezeichnung</t>
   </si>
@@ -309,6 +309,90 @@
   </si>
   <si>
     <t>00092950</t>
+  </si>
+  <si>
+    <t>Film: Antarctica Calling</t>
+  </si>
+  <si>
+    <t>1018.767</t>
+  </si>
+  <si>
+    <t>48257</t>
+  </si>
+  <si>
+    <t>1021.270</t>
+  </si>
+  <si>
+    <t>Film: The Brutalist</t>
+  </si>
+  <si>
+    <t>Universal Pictures International Switzerland GmbH</t>
+  </si>
+  <si>
+    <t>Mühlebachstrasse 54, Zürich 8032 Zürich</t>
+  </si>
+  <si>
+    <t>01 00515 60000 00685 00250 28923</t>
+  </si>
+  <si>
+    <t>2502892</t>
+  </si>
+  <si>
+    <t>1019.343</t>
+  </si>
+  <si>
+    <t>Film: Die Drei ??? - und der Karpatenhund</t>
+  </si>
+  <si>
+    <t>Sony Pictures Releasing Switzerland GmbH</t>
+  </si>
+  <si>
+    <t>Dufourstrasse 24, 8008 Zürich</t>
+  </si>
+  <si>
+    <t>3064757</t>
+  </si>
+  <si>
+    <t>1020.279</t>
+  </si>
+  <si>
+    <t>Film: The Outrun</t>
+  </si>
+  <si>
+    <t>cineworx gmbh</t>
+  </si>
+  <si>
+    <t>Clarastrasse 48, 4005 Basel</t>
+  </si>
+  <si>
+    <t>30 29250 00000 00000 00001 96592</t>
+  </si>
+  <si>
+    <t>19659</t>
+  </si>
+  <si>
+    <t>Film: Prisoners of Fate</t>
+  </si>
+  <si>
+    <t>30 29250 00000 00000 00002 00307</t>
+  </si>
+  <si>
+    <t>20030</t>
+  </si>
+  <si>
+    <t>Weischer Cinema Schweiz GmbH</t>
+  </si>
+  <si>
+    <t>Rämistrasse 6, 8001 Zürich</t>
+  </si>
+  <si>
+    <t>250279TS</t>
+  </si>
+  <si>
+    <t>Weischer Werbeeinnahmen März</t>
+  </si>
+  <si>
+    <t>Weischer Werbeeinnahmen Februar</t>
   </si>
 </sst>
 </file>
@@ -412,8 +496,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{27287C1A-B7AC-49C2-89D9-0074BB2DB80A}"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -460,8 +544,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{895BE82C-25E7-42D8-B99F-BB1A7DC4B1DC}" name="Table3" displayName="Table3" ref="A1:H2" totalsRowShown="0">
-  <autoFilter ref="A1:H2" xr:uid="{895BE82C-25E7-42D8-B99F-BB1A7DC4B1DC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{895BE82C-25E7-42D8-B99F-BB1A7DC4B1DC}" name="Table3" displayName="Table3" ref="A1:H3" totalsRowShown="0">
+  <autoFilter ref="A1:H3" xr:uid="{895BE82C-25E7-42D8-B99F-BB1A7DC4B1DC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H2">
     <sortCondition ref="A1:A2"/>
   </sortState>
@@ -480,8 +564,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K17" totalsRowShown="0">
-  <autoFilter ref="A1:K17" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}" name="Table16" displayName="Table16" ref="A1:K22" totalsRowShown="0">
+  <autoFilter ref="A1:K22" xr:uid="{DECE9D5D-00D4-4490-AE11-80617FB82945}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K4">
     <sortCondition ref="A1:A4"/>
   </sortState>
@@ -495,8 +579,8 @@
     <tableColumn id="4" xr3:uid="{0C538012-5D92-4E64-B81F-85CAF66FE963}" name="Firmennamen"/>
     <tableColumn id="5" xr3:uid="{528DBE91-75A0-4B49-8AC8-06D027A50035}" name="Adresse"/>
     <tableColumn id="6" xr3:uid="{4B5E1481-D849-49CA-8C98-0F7393B356B7}" name="Referenz" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{64D50181-342C-4387-875F-8ADB060C0EDC}" name="Rechnungsnummer" dataDxfId="0"/>
-    <tableColumn id="11" xr3:uid="{9B01639A-96D8-4A50-B1D3-C69E9C49B9DA}" name="Buchungskonto" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{64D50181-342C-4387-875F-8ADB060C0EDC}" name="Rechnungsnummer" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{9B01639A-96D8-4A50-B1D3-C69E9C49B9DA}" name="Buchungskonto" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -526,9 +610,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -566,7 +650,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -672,7 +756,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -822,19 +906,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A72045E-24F3-4DFF-AD02-E9648BA6850D}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" customWidth="1"/>
-    <col min="2" max="2" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="15.42578125" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" customWidth="1"/>
+    <col min="2" max="2" width="37.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.453125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="36" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="42.42578125" customWidth="1"/>
+    <col min="8" max="8" width="42.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -858,6 +942,52 @@
       </c>
       <c r="H1" s="2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" s="4">
+        <v>45755</v>
+      </c>
+      <c r="E2" s="3">
+        <v>6.27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C3" s="4">
+        <v>45692</v>
+      </c>
+      <c r="E3" s="3">
+        <v>7.96</v>
+      </c>
+      <c r="F3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" t="s">
+        <v>114</v>
+      </c>
+      <c r="H3" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -883,22 +1013,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D174BE7-BB11-4664-AEC1-AB301D6C9797}">
   <dimension ref="A1:L114"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="45.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="45.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31" customWidth="1"/>
-    <col min="8" max="8" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.54296875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -933,7 +1063,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -958,7 +1088,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -982,7 +1112,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1005,7 +1135,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1034,7 +1164,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1067,7 +1197,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1102,7 +1232,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1137,7 +1267,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1164,7 +1294,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1199,7 +1329,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1234,7 +1364,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1259,7 +1389,7 @@
       </c>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1294,7 +1424,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1329,7 +1459,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1356,7 +1486,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1385,7 +1515,7 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1420,295 +1550,451 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F18" s="3"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F19" s="3"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F20" s="3"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F21" s="3"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F22" s="3"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1">
+        <v>45739</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="1">
+        <v>45755</v>
+      </c>
+      <c r="F18" s="3">
+        <v>257</v>
+      </c>
+      <c r="G18" t="s">
+        <v>38</v>
+      </c>
+      <c r="H18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="1">
+        <v>45718</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="1">
+        <v>45743</v>
+      </c>
+      <c r="F19" s="3">
+        <v>162.94999999999999</v>
+      </c>
+      <c r="G19" t="s">
+        <v>95</v>
+      </c>
+      <c r="H19" t="s">
+        <v>96</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="1">
+        <v>45690</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D20" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="1">
+        <v>45727</v>
+      </c>
+      <c r="F20" s="3">
+        <v>210.1</v>
+      </c>
+      <c r="G20" t="s">
+        <v>101</v>
+      </c>
+      <c r="H20" t="s">
+        <v>102</v>
+      </c>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="1">
+        <v>45674</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D21" t="s">
+        <v>105</v>
+      </c>
+      <c r="E21" s="1">
+        <v>45758</v>
+      </c>
+      <c r="F21" s="3">
+        <v>205.4</v>
+      </c>
+      <c r="G21" t="s">
+        <v>106</v>
+      </c>
+      <c r="H21" t="s">
+        <v>107</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="1">
+        <v>45738</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D22" t="s">
+        <v>110</v>
+      </c>
+      <c r="E22" s="1">
+        <v>45758</v>
+      </c>
+      <c r="F22" s="3">
+        <v>205.4</v>
+      </c>
+      <c r="G22" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" t="s">
+        <v>107</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F101" s="3"/>
     </row>
-    <row r="102" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F102" s="3"/>
     </row>
-    <row r="103" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F103" s="3"/>
     </row>
-    <row r="104" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F104" s="3"/>
     </row>
-    <row r="105" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F105" s="3"/>
     </row>
-    <row r="106" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F106" s="3"/>
     </row>
-    <row r="107" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F107" s="3"/>
     </row>
-    <row r="108" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F108" s="3"/>
     </row>
-    <row r="109" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F109" s="3"/>
     </row>
-    <row r="110" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F110" s="3"/>
     </row>
-    <row r="111" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F111" s="3"/>
     </row>
-    <row r="112" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F112" s="3"/>
     </row>
-    <row r="113" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F113" s="3"/>
     </row>
-    <row r="114" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="6:6" x14ac:dyDescent="0.35">
       <c r="F114" s="3"/>
     </row>
   </sheetData>
@@ -1742,48 +2028,48 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EFEBA5D-FF22-4032-BB29-794CF56A632B}">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1799,32 +2085,32 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7625BC9-72E3-4F2B-8D7E-DECECAE27301}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>34</v>
       </c>

</xml_diff>